<commit_message>
removed duplicate members, uploaded fixed gephi file
</commit_message>
<xml_diff>
--- a/pre_survey.xlsx
+++ b/pre_survey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilabbe/Documents/GitHub/cdj_networks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B88E81-FC6F-F142-8C9A-E77DA8D4781A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{631DD847-5D2E-0944-8203-C851AC493B4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="103">
   <si>
     <t>ID</t>
   </si>
@@ -230,9 +230,6 @@
     <t>ejt74@cornell.edu</t>
   </si>
   <si>
-    <t>Tu Elinor</t>
-  </si>
-  <si>
     <t>ig276@cornell.edu</t>
   </si>
   <si>
@@ -323,9 +320,6 @@
     <t>ach282@cornell.edu</t>
   </si>
   <si>
-    <t>Hsu, Arianna</t>
-  </si>
-  <si>
     <t>kna42@cornell.edu</t>
   </si>
   <si>
@@ -336,9 +330,6 @@
   </si>
   <si>
     <t>ejl252@cornell.edu</t>
-  </si>
-  <si>
-    <t>Emiline Labbe</t>
   </si>
   <si>
     <t>aaa466@cornell.edu</t>
@@ -407,7 +398,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="53">
+  <dxfs count="52">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -556,9 +547,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
     </dxf>
     <dxf>
@@ -584,14 +572,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:BA42" totalsRowShown="0">
   <autoFilter ref="A1:BA42" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="53">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="49"/>
-    <tableColumn id="53" xr3:uid="{BC717FD1-5508-EC4C-9FF4-8AAFEE9DF844}" name="NetID" dataDxfId="48">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="48"/>
+    <tableColumn id="53" xr3:uid="{BC717FD1-5508-EC4C-9FF4-8AAFEE9DF844}" name="NetID" dataDxfId="47">
       <calculatedColumnFormula>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="46"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Nikhil Chinchalkar" dataDxfId="45"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Jason Wang" dataDxfId="44"/>
@@ -963,7 +951,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1928,7 +1916,7 @@
         <v>ejt74</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" t="s">
@@ -2081,14 +2069,14 @@
         <v>45922.7164583333</v>
       </c>
       <c r="D8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E8" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
         <v>ig276</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" t="s">
@@ -2241,7 +2229,7 @@
         <v>45922.716493055603</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E9" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -2401,7 +2389,7 @@
         <v>45922.716516203698</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -2561,7 +2549,7 @@
         <v>45922.716550925899</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -2721,7 +2709,7 @@
         <v>45922.716574074097</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E12" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -2881,7 +2869,7 @@
         <v>45922.716574074097</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E13" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3041,7 +3029,7 @@
         <v>45922.716608796298</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E14" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3070,7 +3058,7 @@
         <v>56</v>
       </c>
       <c r="N14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O14" t="s">
         <v>59</v>
@@ -3201,7 +3189,7 @@
         <v>45922.716724537</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E15" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3361,7 +3349,7 @@
         <v>45922.7168634259</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E16" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3521,7 +3509,7 @@
         <v>45922.716874999998</v>
       </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3681,7 +3669,7 @@
         <v>45922.716932870397</v>
       </c>
       <c r="D18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E18" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3841,7 +3829,7 @@
         <v>45922.716990740701</v>
       </c>
       <c r="D19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E19" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -3918,10 +3906,10 @@
         <v>56</v>
       </c>
       <c r="AD19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AE19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF19" t="s">
         <v>57</v>
@@ -4001,7 +3989,7 @@
         <v>45922.717060185198</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E20" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -4161,7 +4149,7 @@
         <v>45922.717071759304</v>
       </c>
       <c r="D21" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E21" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -4321,7 +4309,7 @@
         <v>45922.717164351903</v>
       </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E22" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -4481,7 +4469,7 @@
         <v>45922.717164351903</v>
       </c>
       <c r="D23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E23" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -4641,7 +4629,7 @@
         <v>45922.717210648101</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E24" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -4801,7 +4789,7 @@
         <v>45922.717280092598</v>
       </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -4961,7 +4949,7 @@
         <v>45922.717349537001</v>
       </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E26" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -5059,7 +5047,7 @@
         <v>59</v>
       </c>
       <c r="AK26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AL26" t="s">
         <v>59</v>
@@ -5121,14 +5109,14 @@
         <v>45922.717372685198</v>
       </c>
       <c r="D27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E27" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
         <v>ra596</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" t="s">
@@ -5281,7 +5269,7 @@
         <v>45922.717384259297</v>
       </c>
       <c r="D28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E28" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -5441,7 +5429,7 @@
         <v>45922.717453703699</v>
       </c>
       <c r="D29" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E29" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -5601,7 +5589,7 @@
         <v>45922.717546296299</v>
       </c>
       <c r="D30" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E30" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -5761,7 +5749,7 @@
         <v>45922.717569444401</v>
       </c>
       <c r="D31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E31" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -5921,7 +5909,7 @@
         <v>45922.717754629601</v>
       </c>
       <c r="D32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E32" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -6081,7 +6069,7 @@
         <v>45922.717766203699</v>
       </c>
       <c r="D33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E33" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -6241,14 +6229,14 @@
         <v>45922.717870370398</v>
       </c>
       <c r="D34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E34" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
         <v>ach282</v>
       </c>
       <c r="F34" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" t="s">
@@ -6401,7 +6389,7 @@
         <v>45922.717928240701</v>
       </c>
       <c r="D35" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E35" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -6561,7 +6549,7 @@
         <v>45922.719409722202</v>
       </c>
       <c r="D36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E36" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -6581,7 +6569,7 @@
         <v>54</v>
       </c>
       <c r="K36" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L36" t="s">
         <v>54</v>
@@ -6721,7 +6709,7 @@
         <v>45922.734120370398</v>
       </c>
       <c r="D37" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E37" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -6881,14 +6869,14 @@
         <v>45922.7667939815</v>
       </c>
       <c r="D38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E38" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
         <v>ejl252</v>
       </c>
       <c r="F38" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" t="s">
@@ -7041,7 +7029,7 @@
         <v>45922.7975925926</v>
       </c>
       <c r="D39" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E39" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -7201,7 +7189,7 @@
         <v>45922.797708333303</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E40" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -7361,7 +7349,7 @@
         <v>45922.817662037</v>
       </c>
       <c r="D41" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E41" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>
@@ -7521,7 +7509,7 @@
         <v>45922.908483796302</v>
       </c>
       <c r="D42" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E42" t="str">
         <f>LEFT(Table1[[#This Row],[Email]],FIND("@",Table1[[#This Row],[Email]])-1)</f>

</xml_diff>